<commit_message>
chore(weekly-sync): auto-pull through 2026-08-17
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week33.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week33.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SD" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SB" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="SD" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SB" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +36,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -47,21 +44,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,42 +419,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Portfolio name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Advertised ASIN</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>14 Day Total Sales (₹)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>14 Day Total Units (#)</t>
         </is>
@@ -662,10 +650,10 @@
         <v>56117</v>
       </c>
       <c r="G8" t="n">
-        <v>16502.56</v>
+        <v>18874.59</v>
       </c>
       <c r="H8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -1110,10 +1098,10 @@
         <v>40579</v>
       </c>
       <c r="G24" t="n">
-        <v>67866.09</v>
+        <v>71933.03999999999</v>
       </c>
       <c r="H24" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="25">
@@ -1418,10 +1406,10 @@
         <v>10735</v>
       </c>
       <c r="G35" t="n">
-        <v>41855.89999999999</v>
+        <v>46431.32000000001</v>
       </c>
       <c r="H35" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="36">
@@ -1726,10 +1714,10 @@
         <v>8742</v>
       </c>
       <c r="G46" t="n">
-        <v>20542.39</v>
+        <v>23676.28</v>
       </c>
       <c r="H46" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="47">
@@ -1810,10 +1798,10 @@
         <v>66024</v>
       </c>
       <c r="G49" t="n">
-        <v>47705.11</v>
+        <v>39231.38</v>
       </c>
       <c r="H49" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -1863,7 +1851,7 @@
         <v>688</v>
       </c>
       <c r="F51" t="n">
-        <v>61048</v>
+        <v>61047</v>
       </c>
       <c r="G51" t="n">
         <v>8030.5</v>
@@ -1978,10 +1966,10 @@
         <v>7436</v>
       </c>
       <c r="G55" t="n">
-        <v>0</v>
+        <v>4575.42</v>
       </c>
       <c r="H55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -2793,7 +2781,7 @@
         <v>38787.85</v>
       </c>
       <c r="H84" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="85">
@@ -3319,7 +3307,7 @@
         <v>1360</v>
       </c>
       <c r="F103" t="n">
-        <v>143439</v>
+        <v>143438</v>
       </c>
       <c r="G103" t="n">
         <v>25776.26</v>
@@ -3574,10 +3562,10 @@
         <v>65744</v>
       </c>
       <c r="G112" t="n">
-        <v>59379.66</v>
+        <v>50861.86</v>
       </c>
       <c r="H112" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="113">
@@ -3627,13 +3615,13 @@
         <v>326</v>
       </c>
       <c r="F114" t="n">
-        <v>55394</v>
+        <v>55393</v>
       </c>
       <c r="G114" t="n">
-        <v>13970.4</v>
+        <v>14986.5</v>
       </c>
       <c r="H114" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="115">
@@ -3742,10 +3730,10 @@
         <v>164305</v>
       </c>
       <c r="G118" t="n">
-        <v>67867.79000000001</v>
+        <v>72951.69</v>
       </c>
       <c r="H118" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="119">
@@ -4193,7 +4181,7 @@
         <v>8926.280000000001</v>
       </c>
       <c r="H134" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="135">
@@ -4218,10 +4206,10 @@
         <v>43651</v>
       </c>
       <c r="G135" t="n">
-        <v>32099.08</v>
+        <v>30744</v>
       </c>
       <c r="H135" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="136">
@@ -4383,7 +4371,7 @@
         <v>732</v>
       </c>
       <c r="F141" t="n">
-        <v>79599</v>
+        <v>79598</v>
       </c>
       <c r="G141" t="n">
         <v>43134.75</v>
@@ -4607,7 +4595,7 @@
         <v>223</v>
       </c>
       <c r="F149" t="n">
-        <v>151443</v>
+        <v>151442</v>
       </c>
       <c r="G149" t="n">
         <v>10945.76</v>
@@ -4890,10 +4878,10 @@
         <v>15479</v>
       </c>
       <c r="G159" t="n">
-        <v>5083.06</v>
+        <v>7370.35</v>
       </c>
       <c r="H159" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="160">
@@ -5145,7 +5133,7 @@
         <v>14434.75</v>
       </c>
       <c r="H168" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="169">
@@ -5226,10 +5214,10 @@
         <v>81394</v>
       </c>
       <c r="G171" t="n">
-        <v>4144.07</v>
+        <v>6685.6</v>
       </c>
       <c r="H171" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="172">
@@ -5310,10 +5298,10 @@
         <v>6004</v>
       </c>
       <c r="G174" t="n">
-        <v>15272.03</v>
+        <v>12222.03</v>
       </c>
       <c r="H174" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="175">
@@ -5338,10 +5326,10 @@
         <v>10577</v>
       </c>
       <c r="G175" t="n">
-        <v>0</v>
+        <v>7626.27</v>
       </c>
       <c r="H175" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="176">
@@ -5755,7 +5743,7 @@
         <v>186</v>
       </c>
       <c r="F190" t="n">
-        <v>18591</v>
+        <v>18590</v>
       </c>
       <c r="G190" t="n">
         <v>4403.4</v>
@@ -5814,10 +5802,10 @@
         <v>42230</v>
       </c>
       <c r="G192" t="n">
-        <v>13970.4</v>
+        <v>17018.7</v>
       </c>
       <c r="H192" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="193">
@@ -5951,7 +5939,7 @@
         <v>99</v>
       </c>
       <c r="F197" t="n">
-        <v>13088</v>
+        <v>13087</v>
       </c>
       <c r="G197" t="n">
         <v>4573.74</v>
@@ -5979,7 +5967,7 @@
         <v>50</v>
       </c>
       <c r="F198" t="n">
-        <v>5825</v>
+        <v>5824</v>
       </c>
       <c r="G198" t="n">
         <v>0</v>
@@ -6085,13 +6073,13 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>16461.3</v>
+        <v>16446.52</v>
       </c>
       <c r="E202" t="n">
-        <v>1313</v>
+        <v>1312</v>
       </c>
       <c r="F202" t="n">
-        <v>168966</v>
+        <v>168961</v>
       </c>
       <c r="G202" t="n">
         <v>64538.21000000001</v>
@@ -6147,7 +6135,7 @@
         <v>734</v>
       </c>
       <c r="F204" t="n">
-        <v>165917</v>
+        <v>165916</v>
       </c>
       <c r="G204" t="n">
         <v>9864.400000000001</v>
@@ -6626,10 +6614,10 @@
         <v>2018</v>
       </c>
       <c r="G221" t="n">
-        <v>0</v>
+        <v>21862.72</v>
       </c>
       <c r="H221" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="222">
@@ -7774,10 +7762,10 @@
         <v>28699</v>
       </c>
       <c r="G262" t="n">
-        <v>25791.55</v>
+        <v>28163.58</v>
       </c>
       <c r="H262" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="263">
@@ -7914,10 +7902,10 @@
         <v>38276</v>
       </c>
       <c r="G267" t="n">
-        <v>26267.8</v>
+        <v>32622.88</v>
       </c>
       <c r="H267" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="268">
@@ -7970,10 +7958,10 @@
         <v>9631</v>
       </c>
       <c r="G269" t="n">
-        <v>5083.9</v>
+        <v>0</v>
       </c>
       <c r="H269" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="270">
@@ -8194,10 +8182,10 @@
         <v>29497</v>
       </c>
       <c r="G277" t="n">
-        <v>22368.65</v>
+        <v>25588.14</v>
       </c>
       <c r="H277" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="278">
@@ -8303,7 +8291,7 @@
         <v>391</v>
       </c>
       <c r="F281" t="n">
-        <v>71325</v>
+        <v>71324</v>
       </c>
       <c r="G281" t="n">
         <v>15075.38</v>
@@ -8418,10 +8406,10 @@
         <v>23522</v>
       </c>
       <c r="G285" t="n">
-        <v>15469.51</v>
+        <v>17248.32</v>
       </c>
       <c r="H285" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="286">
@@ -8670,10 +8658,10 @@
         <v>4507</v>
       </c>
       <c r="G294" t="n">
-        <v>11767.8</v>
+        <v>8505.940000000001</v>
       </c>
       <c r="H294" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="295">
@@ -8719,42 +8707,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Portfolio name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Advertised ASIN</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>14 Day Total Sales (₹)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>14 Day Total Units (#)</t>
         </is>
@@ -9109,10 +9097,10 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>10843.68</v>
+        <v>10842.78</v>
       </c>
       <c r="E14" t="n">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="F14" t="n">
         <v>217075</v>
@@ -9121,7 +9109,7 @@
         <v>50805.45</v>
       </c>
       <c r="H14" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15">
@@ -9473,19 +9461,19 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1280.12</v>
+        <v>1279.25</v>
       </c>
       <c r="E27" t="n">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="F27" t="n">
         <v>127419</v>
       </c>
       <c r="G27" t="n">
-        <v>14828.81</v>
+        <v>7202.54</v>
       </c>
       <c r="H27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -9697,10 +9685,10 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1068.46</v>
+        <v>1065.42</v>
       </c>
       <c r="E35" t="n">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="F35" t="n">
         <v>46675</v>
@@ -9809,19 +9797,19 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>4202.96</v>
+        <v>4202.29</v>
       </c>
       <c r="E39" t="n">
-        <v>1725</v>
+        <v>1724</v>
       </c>
       <c r="F39" t="n">
         <v>462575</v>
       </c>
       <c r="G39" t="n">
-        <v>12624.58</v>
+        <v>26605.93</v>
       </c>
       <c r="H39" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="40">
@@ -10119,47 +10107,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Portfolio name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Advertised ASIN</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>14 Day Total Sales (₹)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>14 Day Total Units (#)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
@@ -10550,7 +10538,7 @@
         <v>53.53930695422087</v>
       </c>
       <c r="G13" t="n">
-        <v>1426.260055012814</v>
+        <v>1553.167733680186</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -10583,10 +10571,10 @@
         <v>1876.720693045779</v>
       </c>
       <c r="G14" t="n">
-        <v>49994.88994498719</v>
+        <v>54443.40226631982</v>
       </c>
       <c r="H14" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -10607,19 +10595,19 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>9341</v>
+        <v>10877</v>
       </c>
       <c r="E15" t="n">
-        <v>141</v>
+        <v>165</v>
       </c>
       <c r="F15" t="n">
-        <v>1564.175255339063</v>
+        <v>1821.449153824488</v>
       </c>
       <c r="G15" t="n">
-        <v>10038.47979615326</v>
+        <v>11689.5983797059</v>
       </c>
       <c r="H15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -10640,19 +10628,19 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>6975</v>
+        <v>6092</v>
       </c>
       <c r="E16" t="n">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="F16" t="n">
-        <v>1167.963808644794</v>
+        <v>1020.051949274318</v>
       </c>
       <c r="G16" t="n">
-        <v>7495.695290984171</v>
+        <v>6546.434518040841</v>
       </c>
       <c r="H16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -10673,16 +10661,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>5157</v>
+        <v>4504</v>
       </c>
       <c r="E17" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="F17" t="n">
-        <v>863.5609360161423</v>
+        <v>754.1988969011934</v>
       </c>
       <c r="G17" t="n">
-        <v>5542.114912862571</v>
+        <v>4840.257102253258</v>
       </c>
       <c r="H17" t="n">
         <v>3</v>
@@ -10751,7 +10739,7 @@
         <v>6069.634387508736</v>
       </c>
       <c r="H19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -11036,7 +11024,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>78267</v>
+        <v>78266</v>
       </c>
       <c r="E28" t="n">
         <v>778</v>

</xml_diff>